<commit_message>
guardar otro si listo
</commit_message>
<xml_diff>
--- a/storage/plantillas/cargue_otro_si.xlsx
+++ b/storage/plantillas/cargue_otro_si.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ruben-castillo\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\Aescala-laravel\storage\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF3375CD-3106-4FCD-9F5A-B34638F840F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD6955CD-AB81-4752-BCF8-C979D5ECEC13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{45BA13F3-8FAC-44DC-AC95-F914AF6A08A7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{45BA13F3-8FAC-44DC-AC95-F914AF6A08A7}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Pantilla Otro Si" sheetId="1" r:id="rId1"/>
+    <sheet name="Recomendaciones de uso" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="39">
   <si>
     <t>ESPACIO</t>
   </si>
@@ -93,7 +94,342 @@
     <t xml:space="preserve">PROYECTO: </t>
   </si>
   <si>
-    <t>SAUKO - TORRE 2 - APTO 805 MAURICIO URIBE HIGUITA</t>
+    <t>PROYECTO (Fila 1)</t>
+  </si>
+  <si>
+    <t>Campo</t>
+  </si>
+  <si>
+    <t>Descripción</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">En esta celda se debe digitar </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>el nombre exacto del proyecto</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> al que se le realizará el “Otro Sí”. El nombre debe coincidir exactamente con el registrado en el sistema (sin espacios adicionales ni diferencias de mayúsculas o acentos).</t>
+    </r>
+  </si>
+  <si>
+    <t>Encabezado</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Las columnas del encabezado </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>no deben ser modificadas</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (ni el texto ni el orden). Alterar estos valores puede generar errores al momento de cargar el archivo.</t>
+    </r>
+  </si>
+  <si>
+    <t>Espacios (Columna A)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Después del encabezado, en la columna </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> se debe ingresar el nombre del </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Espacio o Área</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (por ejemplo: “COCINA”, “BAÑO PRINCIPAL”, “SALA”). Este nombre debe coincidir exactamente con los registrados en la base de datos. Los ítems siguientes a un espacio pertenecen a dicho espacio hasta que se indique un nuevo nombre en la columna A.</t>
+    </r>
+  </si>
+  <si>
+    <t>MATERIAL / ACTIVIDAD (Columna C)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Este campo es </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>obligatorio</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> para cada fila. Indica la descripción del material, producto o actividad que se va a ejecutar dentro del espacio correspondiente.</t>
+    </r>
+  </si>
+  <si>
+    <t>CANT (Columna D)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Este campo es </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>obligatorio</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> y debe contener un </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>número entero mayor que 0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, que representa la cantidad del material o actividad. No se permiten valores decimales ni negativos.</t>
+    </r>
+  </si>
+  <si>
+    <t>VALOR UNITARIO (Columna E)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Este campo es </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>obligatorio</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> y debe contener un </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>valor numérico entero mayor que 0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. El formato puede incluir símbolo de moneda (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>$</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>) y separadores de miles (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">) — el sistema los normalizará automáticamente. Ejemplo válido: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>$ 350,000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>VALOR TOTAL (Columna F)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Este campo puede dejarse vacío. El sistema calculará automáticamente el valor total como </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>CANT × VALOR UNITARIO</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Filas vacías</t>
+  </si>
+  <si>
+    <t>Las filas completamente vacías serán ignoradas durante el proceso de validación.</t>
+  </si>
+  <si>
+    <t>Recomendación general</t>
+  </si>
+  <si>
+    <t>Verifique cuidadosamente que todos los nombres de proyecto y áreas coincidan exactamente con los registrados en el sistema, y que las cantidades y valores sean correctos antes de realizar el cargue, puedes borra una session especifica siempre i cuando cumplas las recomedaciones.</t>
+  </si>
+  <si>
+    <t>|| Ingrese Nombre del proyecto ||</t>
   </si>
 </sst>
 </file>
@@ -104,7 +440,7 @@
     <numFmt numFmtId="6" formatCode="&quot;$&quot;\ #,##0;[Red]\-&quot;$&quot;\ #,##0"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;\ #,##0"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -158,6 +494,27 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="10">
@@ -216,7 +573,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -237,17 +594,6 @@
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -315,26 +661,6 @@
     </border>
     <border>
       <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right/>
       <top style="thin">
         <color indexed="64"/>
@@ -346,7 +672,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -390,26 +716,65 @@
     <xf numFmtId="6" fontId="6" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -417,58 +782,13 @@
     <xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -788,29 +1108,29 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F40"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="23.28515625" customWidth="1"/>
+    <col min="1" max="1" width="25.28515625" customWidth="1"/>
     <col min="3" max="3" width="85.7109375" customWidth="1"/>
     <col min="4" max="4" width="10.7109375" customWidth="1"/>
     <col min="5" max="5" width="11.7109375" customWidth="1"/>
     <col min="6" max="6" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="39" t="s">
+    <row r="1" spans="1:6" ht="30.75" customHeight="1">
+      <c r="A1" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="39" t="s">
-        <v>18</v>
-      </c>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="40"/>
-    </row>
-    <row r="2" spans="1:6" ht="26.25" x14ac:dyDescent="0.25">
+      <c r="B1" s="31"/>
+      <c r="C1" s="37" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="39"/>
+    </row>
+    <row r="2" spans="1:6" ht="26.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -830,8 +1150,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="32" t="s">
+    <row r="3" spans="1:6">
+      <c r="A3" s="21" t="s">
         <v>14</v>
       </c>
       <c r="B3" s="6">
@@ -849,172 +1169,171 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="34"/>
-      <c r="B4" s="27" t="s">
+    <row r="4" spans="1:6">
+      <c r="A4" s="22"/>
+      <c r="B4" s="6">
+        <v>2</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4">
+        <v>0</v>
+      </c>
+      <c r="E4" s="7">
+        <v>0</v>
+      </c>
+      <c r="F4" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="15" customHeight="1">
+      <c r="A5" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="28"/>
-      <c r="D4" s="28"/>
-      <c r="E4" s="29"/>
-      <c r="F4" s="11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="24"/>
+      <c r="C5" s="24"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="25"/>
+      <c r="F5" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="25.5">
+      <c r="A6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="33" t="s">
+    <row r="7" spans="1:6">
+      <c r="A7" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B7" s="6">
         <v>1</v>
       </c>
-      <c r="C6" s="12"/>
-      <c r="D6" s="38">
-        <v>0</v>
-      </c>
-      <c r="E6" s="13">
-        <v>0</v>
-      </c>
-      <c r="F6" s="13">
-        <f>D6*E6</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="34"/>
-      <c r="B7" s="27" t="s">
+      <c r="C7" s="12"/>
+      <c r="D7" s="17">
+        <v>0</v>
+      </c>
+      <c r="E7" s="13">
+        <v>0</v>
+      </c>
+      <c r="F7" s="13">
+        <f>D7*E7</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="22"/>
+      <c r="B8" s="6">
+        <v>2</v>
+      </c>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4">
+        <v>0</v>
+      </c>
+      <c r="E8" s="7">
+        <v>0</v>
+      </c>
+      <c r="F8" s="7">
+        <f>D8*E8</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="1" customFormat="1" ht="15" customHeight="1">
+      <c r="A9" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="28"/>
-      <c r="D7" s="28"/>
-      <c r="E7" s="29"/>
-      <c r="F7" s="11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" s="1" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B8" s="2" t="s">
+      <c r="B9" s="24"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" s="1" customFormat="1" ht="25.5">
+      <c r="A10" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="F10" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="37" t="s">
+    <row r="11" spans="1:6" s="1" customFormat="1">
+      <c r="A11" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="6">
+      <c r="B11" s="6">
         <v>1</v>
       </c>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12">
-        <v>0</v>
-      </c>
-      <c r="E9" s="5">
-        <v>0</v>
-      </c>
-      <c r="F9" s="13">
-        <f>D9*E9</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="37"/>
-      <c r="B10" s="27" t="s">
+      <c r="C11" s="12"/>
+      <c r="D11" s="12">
+        <v>0</v>
+      </c>
+      <c r="E11" s="5">
+        <v>0</v>
+      </c>
+      <c r="F11" s="13">
+        <f>D11*E11</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" s="1" customFormat="1">
+      <c r="A12" s="22"/>
+      <c r="B12" s="6">
+        <v>2</v>
+      </c>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4">
+        <v>0</v>
+      </c>
+      <c r="E12" s="7">
+        <v>0</v>
+      </c>
+      <c r="F12" s="7">
+        <f>D12*E12</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" s="1" customFormat="1" ht="15" customHeight="1">
+      <c r="A13" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="28"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="29"/>
-      <c r="F10" s="11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" s="1" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12" s="6">
-        <v>1</v>
-      </c>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16">
-        <v>0</v>
-      </c>
-      <c r="E12" s="17">
-        <v>0</v>
-      </c>
-      <c r="F12" s="17">
-        <f>D12*E12</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="36"/>
-      <c r="B13" s="27" t="s">
-        <v>8</v>
-      </c>
-      <c r="C13" s="28"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="29"/>
+      <c r="B13" s="24"/>
+      <c r="C13" s="24"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="25"/>
       <c r="F13" s="11">
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" s="1" customFormat="1" ht="25.5">
       <c r="A14" s="2" t="s">
         <v>0</v>
       </c>
@@ -1030,193 +1349,196 @@
       <c r="E14" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="F14" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="25" t="s">
-        <v>7</v>
+    <row r="15" spans="1:6" s="1" customFormat="1">
+      <c r="A15" s="26" t="s">
+        <v>11</v>
       </c>
       <c r="B15" s="6">
         <v>1</v>
       </c>
-      <c r="C15" s="4"/>
-      <c r="D15" s="8">
-        <v>0</v>
-      </c>
-      <c r="E15" s="7">
-        <v>0</v>
-      </c>
-      <c r="F15" s="7">
+      <c r="C15" s="15"/>
+      <c r="D15" s="15">
+        <v>0</v>
+      </c>
+      <c r="E15" s="16">
+        <v>0</v>
+      </c>
+      <c r="F15" s="16">
         <f>D15*E15</f>
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="26"/>
-      <c r="B16" s="27" t="s">
+    <row r="16" spans="1:6" s="1" customFormat="1">
+      <c r="A16" s="27"/>
+      <c r="B16" s="6">
+        <v>2</v>
+      </c>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4">
+        <v>0</v>
+      </c>
+      <c r="E16" s="7">
+        <v>0</v>
+      </c>
+      <c r="F16" s="7">
+        <f>D16*E16</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="15" customHeight="1">
+      <c r="A17" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="28"/>
-      <c r="D16" s="28"/>
-      <c r="E16" s="29"/>
-      <c r="F16" s="11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="24"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="25.5">
+      <c r="A18" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C18" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D18" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="E18" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="F18" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="30" t="s">
+    <row r="19" spans="1:6">
+      <c r="A19" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="B19" s="6">
+        <v>1</v>
+      </c>
+      <c r="C19" s="4"/>
+      <c r="D19" s="8">
+        <v>0</v>
+      </c>
+      <c r="E19" s="7">
+        <v>0</v>
+      </c>
+      <c r="F19" s="7">
+        <f>D19*E19</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" s="22"/>
+      <c r="B20" s="6">
+        <v>2</v>
+      </c>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4">
+        <v>0</v>
+      </c>
+      <c r="E20" s="7">
+        <v>0</v>
+      </c>
+      <c r="F20" s="7">
+        <f>D20*E20</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="15" customHeight="1">
+      <c r="A21" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="B21" s="24"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="25.5">
+      <c r="A22" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="6">
+      <c r="B23" s="6">
         <v>1</v>
       </c>
-      <c r="C18" s="4"/>
-      <c r="D18" s="8">
-        <v>0</v>
-      </c>
-      <c r="E18" s="7">
-        <v>0</v>
-      </c>
-      <c r="F18" s="7">
-        <f>D18*E18</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="31"/>
-      <c r="B19" s="27" t="s">
+      <c r="C23" s="4"/>
+      <c r="D23" s="8">
+        <v>0</v>
+      </c>
+      <c r="E23" s="7">
+        <v>0</v>
+      </c>
+      <c r="F23" s="7">
+        <f>D23*E23</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" s="29"/>
+      <c r="B24" s="6">
+        <v>2</v>
+      </c>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4">
+        <v>0</v>
+      </c>
+      <c r="E24" s="7">
+        <v>0</v>
+      </c>
+      <c r="F24" s="7">
+        <f>D24*E24</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="15" customHeight="1">
+      <c r="A25" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="C19" s="28"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="29"/>
-      <c r="F19" s="11">
-        <f>SUM(F18:F18)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="24" x14ac:dyDescent="0.25">
-      <c r="A21" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="B21" s="6">
-        <v>1</v>
-      </c>
-      <c r="C21" s="9"/>
-      <c r="D21" s="9">
-        <v>0</v>
-      </c>
-      <c r="E21" s="10">
-        <v>0</v>
-      </c>
-      <c r="F21" s="10">
-        <f>D21*E21</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="27" t="s">
-        <v>8</v>
-      </c>
-      <c r="B22" s="28"/>
-      <c r="C22" s="28"/>
-      <c r="D22" s="28"/>
-      <c r="E22" s="29"/>
-      <c r="F22" s="11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="B24" s="6">
-        <v>1</v>
-      </c>
-      <c r="C24" s="12"/>
-      <c r="D24" s="12">
-        <v>0</v>
-      </c>
-      <c r="E24" s="13">
-        <v>0</v>
-      </c>
-      <c r="F24" s="13">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="27" t="s">
-        <v>8</v>
-      </c>
-      <c r="B25" s="28"/>
-      <c r="C25" s="28"/>
-      <c r="D25" s="28"/>
-      <c r="E25" s="29"/>
-      <c r="F25" s="11"/>
-    </row>
-    <row r="26" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B25" s="24"/>
+      <c r="C25" s="24"/>
+      <c r="D25" s="24"/>
+      <c r="E25" s="25"/>
+      <c r="F25" s="11">
+        <f>SUM(F23:F23)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="25.5">
       <c r="A26" s="2" t="s">
         <v>0</v>
       </c>
@@ -1236,76 +1558,323 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="15" t="s">
-        <v>13</v>
+    <row r="27" spans="1:6">
+      <c r="A27" s="21" t="s">
+        <v>16</v>
       </c>
       <c r="B27" s="6">
         <v>1</v>
       </c>
-      <c r="C27" s="12"/>
-      <c r="D27" s="12">
-        <v>0</v>
-      </c>
-      <c r="E27" s="13">
-        <v>0</v>
-      </c>
-      <c r="F27" s="13">
+      <c r="C27" s="9"/>
+      <c r="D27" s="9">
+        <v>0</v>
+      </c>
+      <c r="E27" s="10">
+        <v>0</v>
+      </c>
+      <c r="F27" s="10">
         <f>D27*E27</f>
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="27" t="s">
+    <row r="28" spans="1:6">
+      <c r="A28" s="22"/>
+      <c r="B28" s="6">
+        <v>2</v>
+      </c>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4">
+        <v>0</v>
+      </c>
+      <c r="E28" s="7">
+        <v>0</v>
+      </c>
+      <c r="F28" s="7">
+        <f>D28*E28</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="15" customHeight="1">
+      <c r="A29" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="B28" s="28"/>
-      <c r="C28" s="28"/>
-      <c r="D28" s="28"/>
-      <c r="E28" s="29"/>
-      <c r="F28" s="11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="22" t="s">
+      <c r="B29" s="24"/>
+      <c r="C29" s="24"/>
+      <c r="D29" s="24"/>
+      <c r="E29" s="25"/>
+      <c r="F29" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="25.5">
+      <c r="A30" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="17.25" customHeight="1">
+      <c r="A31" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="B31" s="6">
+        <v>1</v>
+      </c>
+      <c r="C31" s="12"/>
+      <c r="D31" s="12">
+        <v>0</v>
+      </c>
+      <c r="E31" s="13">
+        <v>0</v>
+      </c>
+      <c r="F31" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="17.25" customHeight="1">
+      <c r="A32" s="22"/>
+      <c r="B32" s="6">
+        <v>2</v>
+      </c>
+      <c r="C32" s="4"/>
+      <c r="D32" s="4">
+        <v>0</v>
+      </c>
+      <c r="E32" s="7">
+        <v>0</v>
+      </c>
+      <c r="F32" s="7">
+        <f>D32*E32</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="B33" s="24"/>
+      <c r="C33" s="24"/>
+      <c r="D33" s="24"/>
+      <c r="E33" s="25"/>
+      <c r="F33" s="11"/>
+    </row>
+    <row r="34" spans="1:6" ht="25.5">
+      <c r="A34" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="B35" s="6">
+        <v>1</v>
+      </c>
+      <c r="C35" s="12"/>
+      <c r="D35" s="12">
+        <v>0</v>
+      </c>
+      <c r="E35" s="13">
+        <v>0</v>
+      </c>
+      <c r="F35" s="13">
+        <f>D35*E35</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36" s="22"/>
+      <c r="B36" s="6">
+        <v>2</v>
+      </c>
+      <c r="C36" s="4"/>
+      <c r="D36" s="4">
+        <v>0</v>
+      </c>
+      <c r="E36" s="7">
+        <v>0</v>
+      </c>
+      <c r="F36" s="7">
+        <f>D36*E36</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="15" customHeight="1">
+      <c r="A37" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="B37" s="24"/>
+      <c r="C37" s="24"/>
+      <c r="D37" s="24"/>
+      <c r="E37" s="25"/>
+      <c r="F37" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="18.75" customHeight="1">
+      <c r="A38" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="B29" s="23"/>
-      <c r="C29" s="23"/>
-      <c r="D29" s="23"/>
-      <c r="E29" s="24"/>
-      <c r="F29" s="14"/>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C30" s="20"/>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C31" s="21"/>
+      <c r="B38" s="35"/>
+      <c r="C38" s="35"/>
+      <c r="D38" s="35"/>
+      <c r="E38" s="36"/>
+      <c r="F38" s="14"/>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="C39" s="32"/>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="C40" s="33"/>
     </row>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="B13:E13"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B10:E10"/>
+  <mergeCells count="22">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C1:F1"/>
-    <mergeCell ref="C30:C31"/>
+    <mergeCell ref="C39:C40"/>
+    <mergeCell ref="A38:E38"/>
     <mergeCell ref="A29:E29"/>
+    <mergeCell ref="A37:E37"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="A13:E13"/>
     <mergeCell ref="A15:A16"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="B19:E19"/>
-    <mergeCell ref="A18:A19"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A23:A24"/>
     <mergeCell ref="A25:E25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="143" scale="60" fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D13B4B8-A5C5-446D-887E-F585F52AA22C}">
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" width="135" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="15.75">
+      <c r="A1" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="20" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="30">
+      <c r="A2" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="30">
+      <c r="A3" s="18" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="45">
+      <c r="A4" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="19" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="30">
+      <c r="A5" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="30">
+      <c r="A6" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="30">
+      <c r="A7" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="30">
+      <c r="A10" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="19" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
ajustes en plantilla otro si
</commit_message>
<xml_diff>
--- a/storage/plantillas/cargue_otro_si.xlsx
+++ b/storage/plantillas/cargue_otro_si.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\Aescala-laravel\storage\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD6955CD-AB81-4752-BCF8-C979D5ECEC13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EA403DB-0A64-472F-9180-21E90B5AFF5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{45BA13F3-8FAC-44DC-AC95-F914AF6A08A7}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="61">
   <si>
     <t>ESPACIO</t>
   </si>
@@ -61,9 +61,6 @@
     <t>VALOR UNITARIO</t>
   </si>
   <si>
-    <t>BAÑO SOCIAL</t>
-  </si>
-  <si>
     <t>SUB TOTAL</t>
   </si>
   <si>
@@ -76,9 +73,6 @@
     <t>ZONA DE ESTAR</t>
   </si>
   <si>
-    <t>HABITACION AUXILIAR</t>
-  </si>
-  <si>
     <t>APTO GENERAL</t>
   </si>
   <si>
@@ -86,9 +80,6 @@
   </si>
   <si>
     <t>BAÑO PRIVADO</t>
-  </si>
-  <si>
-    <t>HABITACION PRINCIPAL</t>
   </si>
   <si>
     <t xml:space="preserve">PROYECTO: </t>
@@ -426,10 +417,85 @@
     <t>Recomendación general</t>
   </si>
   <si>
-    <t>Verifique cuidadosamente que todos los nombres de proyecto y áreas coincidan exactamente con los registrados en el sistema, y que las cantidades y valores sean correctos antes de realizar el cargue, puedes borra una session especifica siempre i cuando cumplas las recomedaciones.</t>
-  </si>
-  <si>
     <t>|| Ingrese Nombre del proyecto ||</t>
+  </si>
+  <si>
+    <t>ALCOBA AUXILIAR 1</t>
+  </si>
+  <si>
+    <t>ALCOBA AUXILIAR 2</t>
+  </si>
+  <si>
+    <t>ALCOBA AUXILIAR 3</t>
+  </si>
+  <si>
+    <t>ALCOBA AUXILIAR 4</t>
+  </si>
+  <si>
+    <t>ALCOBA AUXILIAR 5</t>
+  </si>
+  <si>
+    <t>ALCOBA AUXILIAR 6</t>
+  </si>
+  <si>
+    <t>ALCOBA PRINCIPAL</t>
+  </si>
+  <si>
+    <t>ANTEJARDIN</t>
+  </si>
+  <si>
+    <t>BALCON</t>
+  </si>
+  <si>
+    <t>BAÑO ALCOBA AUXILIAR</t>
+  </si>
+  <si>
+    <t>BAÑO ALCOBA PRINCIPAL</t>
+  </si>
+  <si>
+    <t>BAÑO SOCIAL 1</t>
+  </si>
+  <si>
+    <t>BAÑO SOCIAL 2</t>
+  </si>
+  <si>
+    <t>BAÑO SOCIAL 3</t>
+  </si>
+  <si>
+    <t>COMEDOR</t>
+  </si>
+  <si>
+    <t>ESCALERA</t>
+  </si>
+  <si>
+    <t>FACHADA</t>
+  </si>
+  <si>
+    <t>OBRA BLANCA</t>
+  </si>
+  <si>
+    <t>OBRA CIVIL</t>
+  </si>
+  <si>
+    <t>PASILLO</t>
+  </si>
+  <si>
+    <t>PATIO</t>
+  </si>
+  <si>
+    <t>SALA DE TV</t>
+  </si>
+  <si>
+    <t>TERRAZA</t>
+  </si>
+  <si>
+    <t>ZONA DE ESTUDIO</t>
+  </si>
+  <si>
+    <t>ZONA DE OFICIOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verifique cuidadosamente que todos los nombres de proyecto y áreas coincidan exactamente con los registrados en el sistema, y que las cantidades y valores sean correctos antes de realizar el cargue, puedes borra una session especifica siempre i cuando cumplas las recomedaciones. </t>
   </si>
 </sst>
 </file>
@@ -573,7 +639,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -659,20 +725,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -749,46 +806,40 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1108,7 +1159,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F126"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.28515625" customWidth="1"/>
@@ -1119,16 +1170,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30.75" customHeight="1">
-      <c r="A1" s="30" t="s">
-        <v>17</v>
-      </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="37" t="s">
-        <v>38</v>
-      </c>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="39"/>
+      <c r="A1" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="29"/>
+      <c r="C1" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="32"/>
     </row>
     <row r="2" spans="1:6" ht="26.25">
       <c r="A2" s="2" t="s">
@@ -1152,7 +1203,7 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="21" t="s">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="B3" s="6">
         <v>1</v>
@@ -1187,7 +1238,7 @@
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1">
       <c r="A5" s="23" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B5" s="24"/>
       <c r="C5" s="24"/>
@@ -1219,7 +1270,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="21" t="s">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6">
         <v>1</v>
@@ -1255,7 +1306,7 @@
     </row>
     <row r="9" spans="1:6" s="1" customFormat="1" ht="15" customHeight="1">
       <c r="A9" s="23" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9" s="24"/>
       <c r="C9" s="24"/>
@@ -1287,7 +1338,7 @@
     </row>
     <row r="11" spans="1:6" s="1" customFormat="1">
       <c r="A11" s="21" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="B11" s="6">
         <v>1</v>
@@ -1323,7 +1374,7 @@
     </row>
     <row r="13" spans="1:6" s="1" customFormat="1" ht="15" customHeight="1">
       <c r="A13" s="23" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B13" s="24"/>
       <c r="C13" s="24"/>
@@ -1354,8 +1405,8 @@
       </c>
     </row>
     <row r="15" spans="1:6" s="1" customFormat="1">
-      <c r="A15" s="26" t="s">
-        <v>11</v>
+      <c r="A15" s="36" t="s">
+        <v>38</v>
       </c>
       <c r="B15" s="6">
         <v>1</v>
@@ -1373,7 +1424,7 @@
       </c>
     </row>
     <row r="16" spans="1:6" s="1" customFormat="1">
-      <c r="A16" s="27"/>
+      <c r="A16" s="37"/>
       <c r="B16" s="6">
         <v>2</v>
       </c>
@@ -1391,7 +1442,7 @@
     </row>
     <row r="17" spans="1:6" ht="15" customHeight="1">
       <c r="A17" s="23" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B17" s="24"/>
       <c r="C17" s="24"/>
@@ -1423,7 +1474,7 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="21" t="s">
-        <v>7</v>
+        <v>39</v>
       </c>
       <c r="B19" s="6">
         <v>1</v>
@@ -1459,7 +1510,7 @@
     </row>
     <row r="21" spans="1:6" ht="15" customHeight="1">
       <c r="A21" s="23" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B21" s="24"/>
       <c r="C21" s="24"/>
@@ -1490,8 +1541,8 @@
       </c>
     </row>
     <row r="23" spans="1:6">
-      <c r="A23" s="28" t="s">
-        <v>15</v>
+      <c r="A23" s="26" t="s">
+        <v>40</v>
       </c>
       <c r="B23" s="6">
         <v>1</v>
@@ -1509,7 +1560,7 @@
       </c>
     </row>
     <row r="24" spans="1:6">
-      <c r="A24" s="29"/>
+      <c r="A24" s="27"/>
       <c r="B24" s="6">
         <v>2</v>
       </c>
@@ -1527,7 +1578,7 @@
     </row>
     <row r="25" spans="1:6" ht="15" customHeight="1">
       <c r="A25" s="23" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B25" s="24"/>
       <c r="C25" s="24"/>
@@ -1560,7 +1611,7 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="21" t="s">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="B27" s="6">
         <v>1</v>
@@ -1596,7 +1647,7 @@
     </row>
     <row r="29" spans="1:6" ht="15" customHeight="1">
       <c r="A29" s="23" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B29" s="24"/>
       <c r="C29" s="24"/>
@@ -1628,7 +1679,7 @@
     </row>
     <row r="31" spans="1:6" ht="17.25" customHeight="1">
       <c r="A31" s="21" t="s">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="B31" s="6">
         <v>1</v>
@@ -1663,7 +1714,7 @@
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="23" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B33" s="24"/>
       <c r="C33" s="24"/>
@@ -1693,7 +1744,7 @@
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="21" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B35" s="6">
         <v>1</v>
@@ -1729,7 +1780,7 @@
     </row>
     <row r="37" spans="1:6" ht="15" customHeight="1">
       <c r="A37" s="23" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B37" s="24"/>
       <c r="C37" s="24"/>
@@ -1740,27 +1791,1516 @@
       </c>
     </row>
     <row r="38" spans="1:6" ht="18.75" customHeight="1">
-      <c r="A38" s="34" t="s">
+      <c r="A38" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="B39" s="6">
+        <v>1</v>
+      </c>
+      <c r="C39" s="12"/>
+      <c r="D39" s="12">
+        <v>0</v>
+      </c>
+      <c r="E39" s="13">
+        <v>0</v>
+      </c>
+      <c r="F39" s="13">
+        <f>D39*E39</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="A40" s="22"/>
+      <c r="B40" s="6">
+        <v>2</v>
+      </c>
+      <c r="C40" s="4"/>
+      <c r="D40" s="4">
+        <v>0</v>
+      </c>
+      <c r="E40" s="7">
+        <v>0</v>
+      </c>
+      <c r="F40" s="7">
+        <f>D40*E40</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6">
+      <c r="A41" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B41" s="24"/>
+      <c r="C41" s="24"/>
+      <c r="D41" s="24"/>
+      <c r="E41" s="25"/>
+      <c r="F41" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="25.5">
+      <c r="A42" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
+      <c r="A43" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="B43" s="6">
+        <v>1</v>
+      </c>
+      <c r="C43" s="12"/>
+      <c r="D43" s="12">
+        <v>0</v>
+      </c>
+      <c r="E43" s="13">
+        <v>0</v>
+      </c>
+      <c r="F43" s="13">
+        <f>D43*E43</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6">
+      <c r="A44" s="22"/>
+      <c r="B44" s="6">
+        <v>2</v>
+      </c>
+      <c r="C44" s="4"/>
+      <c r="D44" s="4">
+        <v>0</v>
+      </c>
+      <c r="E44" s="7">
+        <v>0</v>
+      </c>
+      <c r="F44" s="7">
+        <f>D44*E44</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6">
+      <c r="A45" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B45" s="24"/>
+      <c r="C45" s="24"/>
+      <c r="D45" s="24"/>
+      <c r="E45" s="25"/>
+      <c r="F45" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="25.5">
+      <c r="A46" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6">
+      <c r="A47" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="B47" s="6">
+        <v>1</v>
+      </c>
+      <c r="C47" s="12"/>
+      <c r="D47" s="12">
+        <v>0</v>
+      </c>
+      <c r="E47" s="13">
+        <v>0</v>
+      </c>
+      <c r="F47" s="13">
+        <f>D47*E47</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6">
+      <c r="A48" s="22"/>
+      <c r="B48" s="6">
+        <v>2</v>
+      </c>
+      <c r="C48" s="4"/>
+      <c r="D48" s="4">
+        <v>0</v>
+      </c>
+      <c r="E48" s="7">
+        <v>0</v>
+      </c>
+      <c r="F48" s="7">
+        <f>D48*E48</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6">
+      <c r="A49" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B49" s="24"/>
+      <c r="C49" s="24"/>
+      <c r="D49" s="24"/>
+      <c r="E49" s="25"/>
+      <c r="F49" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="25.5">
+      <c r="A50" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6">
+      <c r="A51" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="B51" s="6">
+        <v>1</v>
+      </c>
+      <c r="C51" s="12"/>
+      <c r="D51" s="12">
+        <v>0</v>
+      </c>
+      <c r="E51" s="13">
+        <v>0</v>
+      </c>
+      <c r="F51" s="13">
+        <f>D51*E51</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6">
+      <c r="A52" s="22"/>
+      <c r="B52" s="6">
+        <v>2</v>
+      </c>
+      <c r="C52" s="4"/>
+      <c r="D52" s="4">
+        <v>0</v>
+      </c>
+      <c r="E52" s="7">
+        <v>0</v>
+      </c>
+      <c r="F52" s="7">
+        <f>D52*E52</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6">
+      <c r="A53" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B53" s="24"/>
+      <c r="C53" s="24"/>
+      <c r="D53" s="24"/>
+      <c r="E53" s="25"/>
+      <c r="F53" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" ht="25.5">
+      <c r="A54" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6">
+      <c r="A55" s="21" t="s">
+        <v>46</v>
+      </c>
+      <c r="B55" s="6">
+        <v>1</v>
+      </c>
+      <c r="C55" s="12"/>
+      <c r="D55" s="12">
+        <v>0</v>
+      </c>
+      <c r="E55" s="13">
+        <v>0</v>
+      </c>
+      <c r="F55" s="13">
+        <f>D55*E55</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6">
+      <c r="A56" s="22"/>
+      <c r="B56" s="6">
+        <v>2</v>
+      </c>
+      <c r="C56" s="4"/>
+      <c r="D56" s="4">
+        <v>0</v>
+      </c>
+      <c r="E56" s="7">
+        <v>0</v>
+      </c>
+      <c r="F56" s="7">
+        <f>D56*E56</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6">
+      <c r="A57" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B57" s="24"/>
+      <c r="C57" s="24"/>
+      <c r="D57" s="24"/>
+      <c r="E57" s="25"/>
+      <c r="F57" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" ht="25.5">
+      <c r="A58" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6">
+      <c r="A59" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="B59" s="6">
+        <v>1</v>
+      </c>
+      <c r="C59" s="12"/>
+      <c r="D59" s="12">
+        <v>0</v>
+      </c>
+      <c r="E59" s="13">
+        <v>0</v>
+      </c>
+      <c r="F59" s="13">
+        <f>D59*E59</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6">
+      <c r="A60" s="22"/>
+      <c r="B60" s="6">
+        <v>2</v>
+      </c>
+      <c r="C60" s="4"/>
+      <c r="D60" s="4">
+        <v>0</v>
+      </c>
+      <c r="E60" s="7">
+        <v>0</v>
+      </c>
+      <c r="F60" s="7">
+        <f>D60*E60</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6">
+      <c r="A61" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B61" s="24"/>
+      <c r="C61" s="24"/>
+      <c r="D61" s="24"/>
+      <c r="E61" s="25"/>
+      <c r="F61" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" ht="25.5">
+      <c r="A62" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E62" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6">
+      <c r="A63" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="B63" s="6">
+        <v>1</v>
+      </c>
+      <c r="C63" s="12"/>
+      <c r="D63" s="12">
+        <v>0</v>
+      </c>
+      <c r="E63" s="13">
+        <v>0</v>
+      </c>
+      <c r="F63" s="13">
+        <f>D63*E63</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6">
+      <c r="A64" s="22"/>
+      <c r="B64" s="6">
+        <v>2</v>
+      </c>
+      <c r="C64" s="4"/>
+      <c r="D64" s="4">
+        <v>0</v>
+      </c>
+      <c r="E64" s="7">
+        <v>0</v>
+      </c>
+      <c r="F64" s="7">
+        <f>D64*E64</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6">
+      <c r="A65" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B65" s="24"/>
+      <c r="C65" s="24"/>
+      <c r="D65" s="24"/>
+      <c r="E65" s="25"/>
+      <c r="F65" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" ht="25.5">
+      <c r="A66" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6">
+      <c r="A67" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="B67" s="6">
+        <v>1</v>
+      </c>
+      <c r="C67" s="12"/>
+      <c r="D67" s="12">
+        <v>0</v>
+      </c>
+      <c r="E67" s="13">
+        <v>0</v>
+      </c>
+      <c r="F67" s="13">
+        <f>D67*E67</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6">
+      <c r="A68" s="22"/>
+      <c r="B68" s="6">
+        <v>2</v>
+      </c>
+      <c r="C68" s="4"/>
+      <c r="D68" s="4">
+        <v>0</v>
+      </c>
+      <c r="E68" s="7">
+        <v>0</v>
+      </c>
+      <c r="F68" s="7">
+        <f>D68*E68</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6">
+      <c r="A69" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B69" s="24"/>
+      <c r="C69" s="24"/>
+      <c r="D69" s="24"/>
+      <c r="E69" s="25"/>
+      <c r="F69" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" ht="25.5">
+      <c r="A70" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E70" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6">
+      <c r="A71" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="B71" s="6">
+        <v>1</v>
+      </c>
+      <c r="C71" s="12"/>
+      <c r="D71" s="12">
+        <v>0</v>
+      </c>
+      <c r="E71" s="13">
+        <v>0</v>
+      </c>
+      <c r="F71" s="13">
+        <f>D71*E71</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6">
+      <c r="A72" s="22"/>
+      <c r="B72" s="6">
+        <v>2</v>
+      </c>
+      <c r="C72" s="4"/>
+      <c r="D72" s="4">
+        <v>0</v>
+      </c>
+      <c r="E72" s="7">
+        <v>0</v>
+      </c>
+      <c r="F72" s="7">
+        <f>D72*E72</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6">
+      <c r="A73" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B73" s="24"/>
+      <c r="C73" s="24"/>
+      <c r="D73" s="24"/>
+      <c r="E73" s="25"/>
+      <c r="F73" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" ht="25.5">
+      <c r="A74" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E74" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F74" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6">
+      <c r="A75" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="B75" s="6">
+        <v>1</v>
+      </c>
+      <c r="C75" s="12"/>
+      <c r="D75" s="12">
+        <v>0</v>
+      </c>
+      <c r="E75" s="13">
+        <v>0</v>
+      </c>
+      <c r="F75" s="13">
+        <f>D75*E75</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6">
+      <c r="A76" s="22"/>
+      <c r="B76" s="6">
+        <v>2</v>
+      </c>
+      <c r="C76" s="4"/>
+      <c r="D76" s="4">
+        <v>0</v>
+      </c>
+      <c r="E76" s="7">
+        <v>0</v>
+      </c>
+      <c r="F76" s="7">
+        <f>D76*E76</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6">
+      <c r="A77" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B77" s="24"/>
+      <c r="C77" s="24"/>
+      <c r="D77" s="24"/>
+      <c r="E77" s="25"/>
+      <c r="F77" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" ht="25.5">
+      <c r="A78" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F78" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6">
+      <c r="A79" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="B79" s="6">
+        <v>1</v>
+      </c>
+      <c r="C79" s="12"/>
+      <c r="D79" s="12">
+        <v>0</v>
+      </c>
+      <c r="E79" s="13">
+        <v>0</v>
+      </c>
+      <c r="F79" s="13">
+        <f>D79*E79</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6">
+      <c r="A80" s="22"/>
+      <c r="B80" s="6">
+        <v>2</v>
+      </c>
+      <c r="C80" s="4"/>
+      <c r="D80" s="4">
+        <v>0</v>
+      </c>
+      <c r="E80" s="7">
+        <v>0</v>
+      </c>
+      <c r="F80" s="7">
+        <f>D80*E80</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6">
+      <c r="A81" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B81" s="24"/>
+      <c r="C81" s="24"/>
+      <c r="D81" s="24"/>
+      <c r="E81" s="25"/>
+      <c r="F81" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" ht="25.5">
+      <c r="A82" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E82" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F82" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6">
+      <c r="A83" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="B83" s="6">
+        <v>1</v>
+      </c>
+      <c r="C83" s="12"/>
+      <c r="D83" s="12">
+        <v>0</v>
+      </c>
+      <c r="E83" s="13">
+        <v>0</v>
+      </c>
+      <c r="F83" s="13">
+        <f>D83*E83</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6">
+      <c r="A84" s="22"/>
+      <c r="B84" s="6">
+        <v>2</v>
+      </c>
+      <c r="C84" s="4"/>
+      <c r="D84" s="4">
+        <v>0</v>
+      </c>
+      <c r="E84" s="7">
+        <v>0</v>
+      </c>
+      <c r="F84" s="7">
+        <f>D84*E84</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6">
+      <c r="A85" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B85" s="24"/>
+      <c r="C85" s="24"/>
+      <c r="D85" s="24"/>
+      <c r="E85" s="25"/>
+      <c r="F85" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" ht="25.5">
+      <c r="A86" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E86" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F86" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6">
+      <c r="A87" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="B87" s="6">
+        <v>1</v>
+      </c>
+      <c r="C87" s="12"/>
+      <c r="D87" s="12">
+        <v>0</v>
+      </c>
+      <c r="E87" s="13">
+        <v>0</v>
+      </c>
+      <c r="F87" s="13">
+        <f>D87*E87</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6">
+      <c r="A88" s="22"/>
+      <c r="B88" s="6">
+        <v>2</v>
+      </c>
+      <c r="C88" s="4"/>
+      <c r="D88" s="4">
+        <v>0</v>
+      </c>
+      <c r="E88" s="7">
+        <v>0</v>
+      </c>
+      <c r="F88" s="7">
+        <f>D88*E88</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6">
+      <c r="A89" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B89" s="24"/>
+      <c r="C89" s="24"/>
+      <c r="D89" s="24"/>
+      <c r="E89" s="25"/>
+      <c r="F89" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" ht="25.5">
+      <c r="A90" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E90" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F90" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6">
+      <c r="A91" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="B91" s="6">
+        <v>1</v>
+      </c>
+      <c r="C91" s="12"/>
+      <c r="D91" s="12">
+        <v>0</v>
+      </c>
+      <c r="E91" s="13">
+        <v>0</v>
+      </c>
+      <c r="F91" s="13">
+        <f>D91*E91</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6">
+      <c r="A92" s="22"/>
+      <c r="B92" s="6">
+        <v>2</v>
+      </c>
+      <c r="C92" s="4"/>
+      <c r="D92" s="4">
+        <v>0</v>
+      </c>
+      <c r="E92" s="7">
+        <v>0</v>
+      </c>
+      <c r="F92" s="7">
+        <f>D92*E92</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6">
+      <c r="A93" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B93" s="24"/>
+      <c r="C93" s="24"/>
+      <c r="D93" s="24"/>
+      <c r="E93" s="25"/>
+      <c r="F93" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" ht="25.5">
+      <c r="A94" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E94" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F94" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6">
+      <c r="A95" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="B95" s="6">
+        <v>1</v>
+      </c>
+      <c r="C95" s="12"/>
+      <c r="D95" s="12">
+        <v>0</v>
+      </c>
+      <c r="E95" s="13">
+        <v>0</v>
+      </c>
+      <c r="F95" s="13">
+        <f>D95*E95</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6">
+      <c r="A96" s="22"/>
+      <c r="B96" s="6">
+        <v>2</v>
+      </c>
+      <c r="C96" s="4"/>
+      <c r="D96" s="4">
+        <v>0</v>
+      </c>
+      <c r="E96" s="7">
+        <v>0</v>
+      </c>
+      <c r="F96" s="7">
+        <f>D96*E96</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6">
+      <c r="A97" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B97" s="24"/>
+      <c r="C97" s="24"/>
+      <c r="D97" s="24"/>
+      <c r="E97" s="25"/>
+      <c r="F97" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" ht="25.5">
+      <c r="A98" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E98" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F98" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6">
+      <c r="A99" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="B99" s="6">
+        <v>1</v>
+      </c>
+      <c r="C99" s="12"/>
+      <c r="D99" s="12">
+        <v>0</v>
+      </c>
+      <c r="E99" s="13">
+        <v>0</v>
+      </c>
+      <c r="F99" s="13">
+        <f>D99*E99</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6">
+      <c r="A100" s="22"/>
+      <c r="B100" s="6">
+        <v>2</v>
+      </c>
+      <c r="C100" s="4"/>
+      <c r="D100" s="4">
+        <v>0</v>
+      </c>
+      <c r="E100" s="7">
+        <v>0</v>
+      </c>
+      <c r="F100" s="7">
+        <f>D100*E100</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6">
+      <c r="A101" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B101" s="24"/>
+      <c r="C101" s="24"/>
+      <c r="D101" s="24"/>
+      <c r="E101" s="25"/>
+      <c r="F101" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" ht="25.5">
+      <c r="A102" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E102" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F102" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6">
+      <c r="A103" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="B103" s="6">
+        <v>1</v>
+      </c>
+      <c r="C103" s="12"/>
+      <c r="D103" s="12">
+        <v>0</v>
+      </c>
+      <c r="E103" s="13">
+        <v>0</v>
+      </c>
+      <c r="F103" s="13">
+        <f>D103*E103</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6">
+      <c r="A104" s="22"/>
+      <c r="B104" s="6">
+        <v>2</v>
+      </c>
+      <c r="C104" s="4"/>
+      <c r="D104" s="4">
+        <v>0</v>
+      </c>
+      <c r="E104" s="7">
+        <v>0</v>
+      </c>
+      <c r="F104" s="7">
+        <f>D104*E104</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6">
+      <c r="A105" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B105" s="24"/>
+      <c r="C105" s="24"/>
+      <c r="D105" s="24"/>
+      <c r="E105" s="25"/>
+      <c r="F105" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" ht="25.5">
+      <c r="A106" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D106" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E106" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F106" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6">
+      <c r="A107" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="B107" s="6">
+        <v>1</v>
+      </c>
+      <c r="C107" s="12"/>
+      <c r="D107" s="12">
+        <v>0</v>
+      </c>
+      <c r="E107" s="13">
+        <v>0</v>
+      </c>
+      <c r="F107" s="13">
+        <f>D107*E107</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6">
+      <c r="A108" s="22"/>
+      <c r="B108" s="6">
+        <v>2</v>
+      </c>
+      <c r="C108" s="4"/>
+      <c r="D108" s="4">
+        <v>0</v>
+      </c>
+      <c r="E108" s="7">
+        <v>0</v>
+      </c>
+      <c r="F108" s="7">
+        <f>D108*E108</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6">
+      <c r="A109" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B109" s="24"/>
+      <c r="C109" s="24"/>
+      <c r="D109" s="24"/>
+      <c r="E109" s="25"/>
+      <c r="F109" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" ht="25.5">
+      <c r="A110" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B110" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C110" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D110" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E110" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F110" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6">
+      <c r="A111" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="B111" s="6">
+        <v>1</v>
+      </c>
+      <c r="C111" s="12"/>
+      <c r="D111" s="12">
+        <v>0</v>
+      </c>
+      <c r="E111" s="13">
+        <v>0</v>
+      </c>
+      <c r="F111" s="13">
+        <f>D111*E111</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6">
+      <c r="A112" s="22"/>
+      <c r="B112" s="6">
+        <v>2</v>
+      </c>
+      <c r="C112" s="4"/>
+      <c r="D112" s="4">
+        <v>0</v>
+      </c>
+      <c r="E112" s="7">
+        <v>0</v>
+      </c>
+      <c r="F112" s="7">
+        <f>D112*E112</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6">
+      <c r="A113" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B113" s="24"/>
+      <c r="C113" s="24"/>
+      <c r="D113" s="24"/>
+      <c r="E113" s="25"/>
+      <c r="F113" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" ht="25.5">
+      <c r="A114" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B114" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C114" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D114" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E114" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F114" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6">
+      <c r="A115" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="B115" s="6">
+        <v>1</v>
+      </c>
+      <c r="C115" s="12"/>
+      <c r="D115" s="12">
+        <v>0</v>
+      </c>
+      <c r="E115" s="13">
+        <v>0</v>
+      </c>
+      <c r="F115" s="13">
+        <f>D115*E115</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6">
+      <c r="A116" s="22"/>
+      <c r="B116" s="6">
+        <v>2</v>
+      </c>
+      <c r="C116" s="4"/>
+      <c r="D116" s="4">
+        <v>0</v>
+      </c>
+      <c r="E116" s="7">
+        <v>0</v>
+      </c>
+      <c r="F116" s="7">
+        <f>D116*E116</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6">
+      <c r="A117" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B117" s="24"/>
+      <c r="C117" s="24"/>
+      <c r="D117" s="24"/>
+      <c r="E117" s="25"/>
+      <c r="F117" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" ht="25.5">
+      <c r="A118" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B118" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C118" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D118" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E118" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F118" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6">
+      <c r="A119" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="B119" s="6">
+        <v>1</v>
+      </c>
+      <c r="C119" s="12"/>
+      <c r="D119" s="12">
+        <v>0</v>
+      </c>
+      <c r="E119" s="13">
+        <v>0</v>
+      </c>
+      <c r="F119" s="13">
+        <f>D119*E119</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6">
+      <c r="A120" s="22"/>
+      <c r="B120" s="6">
+        <v>2</v>
+      </c>
+      <c r="C120" s="4"/>
+      <c r="D120" s="4">
+        <v>0</v>
+      </c>
+      <c r="E120" s="7">
+        <v>0</v>
+      </c>
+      <c r="F120" s="7">
+        <f>D120*E120</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6">
+      <c r="A121" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B121" s="24"/>
+      <c r="C121" s="24"/>
+      <c r="D121" s="24"/>
+      <c r="E121" s="25"/>
+      <c r="F121" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" ht="25.5">
+      <c r="A122" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B122" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C122" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D122" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E122" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F122" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6">
+      <c r="A123" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="B123" s="6">
+        <v>1</v>
+      </c>
+      <c r="C123" s="12"/>
+      <c r="D123" s="12">
+        <v>0</v>
+      </c>
+      <c r="E123" s="13">
+        <v>0</v>
+      </c>
+      <c r="F123" s="13">
+        <f>D123*E123</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6">
+      <c r="A124" s="22"/>
+      <c r="B124" s="6">
+        <v>2</v>
+      </c>
+      <c r="C124" s="4"/>
+      <c r="D124" s="4">
+        <v>0</v>
+      </c>
+      <c r="E124" s="7">
+        <v>0</v>
+      </c>
+      <c r="F124" s="7">
+        <f>D124*E124</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6">
+      <c r="A125" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B125" s="24"/>
+      <c r="C125" s="24"/>
+      <c r="D125" s="24"/>
+      <c r="E125" s="25"/>
+      <c r="F125" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6">
+      <c r="A126" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="B38" s="35"/>
-      <c r="C38" s="35"/>
-      <c r="D38" s="35"/>
-      <c r="E38" s="36"/>
-      <c r="F38" s="14"/>
-    </row>
-    <row r="39" spans="1:6">
-      <c r="C39" s="32"/>
-    </row>
-    <row r="40" spans="1:6">
-      <c r="C40" s="33"/>
+      <c r="B126" s="34"/>
+      <c r="C126" s="34"/>
+      <c r="D126" s="34"/>
+      <c r="E126" s="35"/>
+      <c r="F126" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="65">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C1:F1"/>
-    <mergeCell ref="C39:C40"/>
-    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="A126:E126"/>
     <mergeCell ref="A29:E29"/>
     <mergeCell ref="A37:E37"/>
     <mergeCell ref="A5:E5"/>
@@ -1779,6 +3319,50 @@
     <mergeCell ref="A11:A12"/>
     <mergeCell ref="A23:A24"/>
     <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="A41:E41"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="A45:E45"/>
+    <mergeCell ref="A47:A48"/>
+    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="A51:A52"/>
+    <mergeCell ref="A53:E53"/>
+    <mergeCell ref="A55:A56"/>
+    <mergeCell ref="A57:E57"/>
+    <mergeCell ref="A59:A60"/>
+    <mergeCell ref="A61:E61"/>
+    <mergeCell ref="A63:A64"/>
+    <mergeCell ref="A65:E65"/>
+    <mergeCell ref="A67:A68"/>
+    <mergeCell ref="A69:E69"/>
+    <mergeCell ref="A71:A72"/>
+    <mergeCell ref="A73:E73"/>
+    <mergeCell ref="A75:A76"/>
+    <mergeCell ref="A77:E77"/>
+    <mergeCell ref="A79:A80"/>
+    <mergeCell ref="A81:E81"/>
+    <mergeCell ref="A83:A84"/>
+    <mergeCell ref="A85:E85"/>
+    <mergeCell ref="A87:A88"/>
+    <mergeCell ref="A89:E89"/>
+    <mergeCell ref="A91:A92"/>
+    <mergeCell ref="A93:E93"/>
+    <mergeCell ref="A95:A96"/>
+    <mergeCell ref="A97:E97"/>
+    <mergeCell ref="A99:A100"/>
+    <mergeCell ref="A101:E101"/>
+    <mergeCell ref="A103:A104"/>
+    <mergeCell ref="A105:E105"/>
+    <mergeCell ref="A107:A108"/>
+    <mergeCell ref="A119:A120"/>
+    <mergeCell ref="A121:E121"/>
+    <mergeCell ref="A123:A124"/>
+    <mergeCell ref="A125:E125"/>
+    <mergeCell ref="A109:E109"/>
+    <mergeCell ref="A111:A112"/>
+    <mergeCell ref="A113:E113"/>
+    <mergeCell ref="A115:A116"/>
+    <mergeCell ref="A117:E117"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="143" scale="60" fitToHeight="0" orientation="portrait" r:id="rId1"/>
@@ -1796,82 +3380,82 @@
   <sheetData>
     <row r="1" spans="1:2" ht="15.75">
       <c r="A1" s="20" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B1" s="20" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="30">
       <c r="A2" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="19" t="s">
         <v>18</v>
-      </c>
-      <c r="B2" s="19" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="30">
       <c r="A3" s="18" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="45">
       <c r="A4" s="18" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="30">
       <c r="A5" s="18" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="30">
       <c r="A6" s="18" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="30">
       <c r="A7" s="18" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="18" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="18" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="30">
       <c r="A10" s="18" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>37</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>